<commit_message>
chore: update Excel files for arbitrage and Geneva odds
</commit_message>
<xml_diff>
--- a/arbitrage_final_report.xlsx
+++ b/arbitrage_final_report.xlsx
@@ -451,22 +451,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lorenzo Sonego vs Edas Butvilas</t>
+          <t>Jenson Brooksby vs Casper Ruud</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PAF Home / Veikkaus Away</t>
+          <t>Veikkaus Home / PAF Away</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.72</v>
+        <v>5.6</v>
       </c>
       <c r="D2" t="n">
-        <v>2.2</v>
+        <v>1.15</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0359</v>
+        <v>1.0481</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -477,22 +477,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jenson Brooksby vs Casper Ruud</t>
+          <t>Lorenzo Sonego vs Edas Butvilas</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Veikkaus Home / PAF Away</t>
+          <t>PAF Home / Veikkaus Away</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5.6</v>
+        <v>2.12</v>
       </c>
       <c r="D3" t="n">
-        <v>1.15</v>
+        <v>1.73</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0481</v>
+        <v>1.0497</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -503,7 +503,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nishesh Basavareddy vs Jaume Munar</t>
+          <t>Alexei Popyrin vs Clement Tabur</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -512,13 +512,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2.55</v>
+        <v>1.45</v>
       </c>
       <c r="D4" t="n">
-        <v>1.51</v>
+        <v>2.76</v>
       </c>
       <c r="E4" t="n">
-        <v>1.0544</v>
+        <v>1.052</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -529,7 +529,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Adrian Mannarino vs Raphael Collignon</t>
+          <t>Nishesh Basavareddy vs Jaume Munar</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -538,13 +538,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>2.55</v>
       </c>
       <c r="D5" t="n">
-        <v>1.06</v>
+        <v>1.51</v>
       </c>
       <c r="E5" t="n">
-        <v>1.0545</v>
+        <v>1.0544</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -555,7 +555,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cameron Norrie vs Mariano Navone</t>
+          <t>Adrian Mannarino vs Raphael Collignon</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,13 +564,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2.12</v>
+        <v>9</v>
       </c>
       <c r="D6" t="n">
-        <v>1.7</v>
+        <v>1.06</v>
       </c>
       <c r="E6" t="n">
-        <v>1.0599</v>
+        <v>1.0545</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -581,7 +581,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Alexei Popyrin vs Clement Tabur</t>
+          <t>Cameron Norrie vs Mariano Navone</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -590,13 +590,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.45</v>
+        <v>2.12</v>
       </c>
       <c r="D7" t="n">
-        <v>2.7</v>
+        <v>1.7</v>
       </c>
       <c r="E7" t="n">
-        <v>1.06</v>
+        <v>1.0599</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>

</xml_diff>